<commit_message>
Ready module reports.py and tests. Fixes dogstring, annotations and different module
</commit_message>
<xml_diff>
--- a/data/operations.xlsx
+++ b/data/operations.xlsx
@@ -1,26 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PyPractice\Analysis_Of_Banking_Transactions\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NikitaK\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E0071C-10A6-40C9-B63A-5BD0B83B99A0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{23A74A38-23F8-43D2-B0D3-22052E0529F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Отчет по операциям" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="827" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="855" uniqueCount="120">
   <si>
     <t>Дата операции</t>
   </si>
@@ -433,7 +439,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -449,9 +455,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Тема Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Стандартная">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -489,7 +495,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Стандартная">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -595,7 +601,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Стандартная">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -745,27 +751,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O126"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:O130"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="19" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="37.109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="26" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="30.6640625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="32" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -812,7 +818,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>45777.771273148152</v>
       </c>
@@ -859,7 +865,7 @@
         <v>-329.99</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>45777.719618055555</v>
       </c>
@@ -906,7 +912,7 @@
         <v>-575</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>45776.939131944448</v>
       </c>
@@ -947,7 +953,7 @@
         <v>-300</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>45776.90152777778</v>
       </c>
@@ -991,7 +997,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>45776.852118055554</v>
       </c>
@@ -1038,7 +1044,7 @@
         <v>-159</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>45776.346377314818</v>
       </c>
@@ -1082,7 +1088,7 @@
         <v>-22874.59</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>45775.859120370369</v>
       </c>
@@ -1129,7 +1135,7 @@
         <v>-159</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>45775.857094907406</v>
       </c>
@@ -1176,7 +1182,7 @@
         <v>-748.96</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>45775.700532407405</v>
       </c>
@@ -1220,7 +1226,7 @@
         <v>50000</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>45775.048958333333</v>
       </c>
@@ -1267,7 +1273,7 @@
         <v>-999.56</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
         <v>45774.578368055554</v>
       </c>
@@ -1311,7 +1317,7 @@
         <v>-70</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
         <v>45774.564201388886</v>
       </c>
@@ -1358,7 +1364,7 @@
         <v>-400</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>45774.563831018517</v>
       </c>
@@ -1405,7 +1411,7 @@
         <v>-1186.93</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>45774.032673611109</v>
       </c>
@@ -1449,7 +1455,7 @@
         <v>-128000</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>45774.031388888892</v>
       </c>
@@ -1490,7 +1496,7 @@
         <v>60000</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>45774.031377314815</v>
       </c>
@@ -1534,7 +1540,7 @@
         <v>-60000</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>45773.726377314815</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>-524.96</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>45773.705266203702</v>
       </c>
@@ -1628,7 +1634,7 @@
         <v>-150</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>45773.686990740738</v>
       </c>
@@ -1675,7 +1681,7 @@
         <v>-999.56</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>45773.666446759256</v>
       </c>
@@ -1716,7 +1722,7 @@
         <v>20000</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>45773.643958333334</v>
       </c>
@@ -1757,7 +1763,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>45773.643946759257</v>
       </c>
@@ -1801,7 +1807,7 @@
         <v>-600</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>45773.63722222222</v>
       </c>
@@ -1848,7 +1854,7 @@
         <v>-210</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>45773.630856481483</v>
       </c>
@@ -1895,7 +1901,7 @@
         <v>-515</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>45773.458680555559</v>
       </c>
@@ -1942,7 +1948,7 @@
         <v>-249</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>45773.450300925928</v>
       </c>
@@ -1989,7 +1995,7 @@
         <v>-325</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>45773.406597222223</v>
       </c>
@@ -2033,7 +2039,7 @@
         <v>-1390</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>45773.333240740743</v>
       </c>
@@ -2071,7 +2077,7 @@
         <v>17800</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>45772.619803240741</v>
       </c>
@@ -2109,7 +2115,7 @@
         <v>4585</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>45772.606782407405</v>
       </c>
@@ -2156,7 +2162,7 @@
         <v>-662</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>45772.443124999998</v>
       </c>
@@ -2203,7 +2209,7 @@
         <v>-665</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>45771.668692129628</v>
       </c>
@@ -2244,7 +2250,7 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A34" s="2">
         <v>45771.654282407406</v>
       </c>
@@ -2285,7 +2291,7 @@
         <v>-6875</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A35" s="2">
         <v>45771.569537037038</v>
       </c>
@@ -2326,7 +2332,7 @@
         <v>-318.99</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
         <v>45771.488576388889</v>
       </c>
@@ -2373,7 +2379,7 @@
         <v>-3295.83</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>45770.99496527778</v>
       </c>
@@ -2420,7 +2426,7 @@
         <v>-502</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>45770.902881944443</v>
       </c>
@@ -2464,7 +2470,7 @@
         <v>-750</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>45770.783877314818</v>
       </c>
@@ -2511,7 +2517,7 @@
         <v>-599</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A40" s="2">
         <v>45770.391643518517</v>
       </c>
@@ -2552,7 +2558,7 @@
         <v>-1125</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>45770.387476851851</v>
       </c>
@@ -2593,7 +2599,7 @@
         <v>-1125</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A42" s="2">
         <v>45769.166620370372</v>
       </c>
@@ -2637,7 +2643,7 @@
         <v>-3000</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>45768.940347222226</v>
       </c>
@@ -2675,7 +2681,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="2">
         <v>45766.713125000002</v>
       </c>
@@ -2713,7 +2719,7 @@
         <v>2700</v>
       </c>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>45766.709224537037</v>
       </c>
@@ -2751,7 +2757,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="2">
         <v>45765.944305555553</v>
       </c>
@@ -2789,7 +2795,7 @@
         <v>160.08000000000001</v>
       </c>
     </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>45765</v>
       </c>
@@ -2824,7 +2830,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>45765</v>
       </c>
@@ -2859,7 +2865,7 @@
         <v>-202.46</v>
       </c>
     </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>45762.945937500001</v>
       </c>
@@ -2897,7 +2903,7 @@
         <v>19.64</v>
       </c>
     </row>
-    <row r="50" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>45762.233449074076</v>
       </c>
@@ -2941,7 +2947,7 @@
         <v>-1000</v>
       </c>
     </row>
-    <row r="51" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>45762.137094907404</v>
       </c>
@@ -2985,7 +2991,7 @@
         <v>-4000</v>
       </c>
     </row>
-    <row r="52" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A52" s="2">
         <v>45762.135775462964</v>
       </c>
@@ -3029,7 +3035,7 @@
         <v>-4874</v>
       </c>
     </row>
-    <row r="53" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>45759.455104166664</v>
       </c>
@@ -3076,7 +3082,7 @@
         <v>-399</v>
       </c>
     </row>
-    <row r="54" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>45757.811041666668</v>
       </c>
@@ -3120,7 +3126,7 @@
         <v>-20000</v>
       </c>
     </row>
-    <row r="55" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A55" s="2">
         <v>45757.800821759258</v>
       </c>
@@ -3164,7 +3170,7 @@
         <v>-5000</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>45757.793321759258</v>
       </c>
@@ -3208,7 +3214,7 @@
         <v>-15000</v>
       </c>
     </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A57" s="2">
         <v>45757.510081018518</v>
       </c>
@@ -3246,7 +3252,7 @@
         <v>68948.179999999993</v>
       </c>
     </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A58" s="2">
         <v>45757.490578703706</v>
       </c>
@@ -3290,7 +3296,7 @@
         <v>-199.69</v>
       </c>
     </row>
-    <row r="59" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="2">
         <v>45757.164120370369</v>
       </c>
@@ -3334,7 +3340,7 @@
         <v>-2500</v>
       </c>
     </row>
-    <row r="60" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>45756.902199074073</v>
       </c>
@@ -3378,7 +3384,7 @@
         <v>-1939</v>
       </c>
     </row>
-    <row r="61" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>45756.897453703707</v>
       </c>
@@ -3422,7 +3428,7 @@
         <v>-139.97999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="2">
         <v>45756.881469907406</v>
       </c>
@@ -3466,7 +3472,7 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="2">
         <v>45756.881111111114</v>
       </c>
@@ -3510,7 +3516,7 @@
         <v>-1180</v>
       </c>
     </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>45756.796851851854</v>
       </c>
@@ -3554,7 +3560,7 @@
         <v>-1800</v>
       </c>
     </row>
-    <row r="65" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>45756.72215277778</v>
       </c>
@@ -3598,7 +3604,7 @@
         <v>-4445</v>
       </c>
     </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A66" s="2">
         <v>45756.630497685182</v>
       </c>
@@ -3642,7 +3648,7 @@
         <v>-3393</v>
       </c>
     </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>45756.560972222222</v>
       </c>
@@ -3686,7 +3692,7 @@
         <v>-840</v>
       </c>
     </row>
-    <row r="68" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A68" s="2">
         <v>45756.412476851852</v>
       </c>
@@ -3730,7 +3736,7 @@
         <v>-14</v>
       </c>
     </row>
-    <row r="69" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A69" s="2">
         <v>45756.359479166669</v>
       </c>
@@ -3774,7 +3780,7 @@
         <v>-1089.95</v>
       </c>
     </row>
-    <row r="70" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A70" s="2">
         <v>45755.941550925927</v>
       </c>
@@ -3809,7 +3815,7 @@
         <v>517.70000000000005</v>
       </c>
     </row>
-    <row r="71" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A71" s="2">
         <v>45755.708425925928</v>
       </c>
@@ -3850,7 +3856,7 @@
         <v>-1100</v>
       </c>
     </row>
-    <row r="72" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="2">
         <v>45755.676122685189</v>
       </c>
@@ -3888,7 +3894,7 @@
         <v>49099.24</v>
       </c>
     </row>
-    <row r="73" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>45755.662245370368</v>
       </c>
@@ -3929,7 +3935,7 @@
         <v>-810</v>
       </c>
     </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A74" s="2">
         <v>45755.067754629628</v>
       </c>
@@ -3970,7 +3976,7 @@
         <v>-550</v>
       </c>
     </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A75" s="2">
         <v>45754.866030092591</v>
       </c>
@@ -4011,7 +4017,7 @@
         <v>-400</v>
       </c>
     </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>45754.736122685186</v>
       </c>
@@ -4052,7 +4058,7 @@
         <v>-450</v>
       </c>
     </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A77" s="2">
         <v>45754.563379629632</v>
       </c>
@@ -4096,7 +4102,7 @@
         <v>-530</v>
       </c>
     </row>
-    <row r="78" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A78" s="2">
         <v>45754.054363425923</v>
       </c>
@@ -4137,7 +4143,7 @@
         <v>-150</v>
       </c>
     </row>
-    <row r="79" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>45753.961631944447</v>
       </c>
@@ -4181,7 +4187,7 @@
         <v>-430.18</v>
       </c>
     </row>
-    <row r="80" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>45753.956736111111</v>
       </c>
@@ -4222,7 +4228,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="81" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A81" s="2">
         <v>45753.956724537034</v>
       </c>
@@ -4266,7 +4272,7 @@
         <v>-1000</v>
       </c>
     </row>
-    <row r="82" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A82" s="2">
         <v>45753.765706018516</v>
       </c>
@@ -4307,7 +4313,7 @@
         <v>-1000</v>
       </c>
     </row>
-    <row r="83" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>45753.746689814812</v>
       </c>
@@ -4348,7 +4354,7 @@
         <v>-10</v>
       </c>
     </row>
-    <row r="84" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>45753.73846064815</v>
       </c>
@@ -4389,7 +4395,7 @@
         <v>9.33</v>
       </c>
     </row>
-    <row r="85" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>45753.73846064815</v>
       </c>
@@ -4433,7 +4439,7 @@
         <v>-9.33</v>
       </c>
     </row>
-    <row r="86" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>45753.738344907404</v>
       </c>
@@ -4474,7 +4480,7 @@
         <v>613.54</v>
       </c>
     </row>
-    <row r="87" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A87" s="2">
         <v>45753.738333333335</v>
       </c>
@@ -4518,7 +4524,7 @@
         <v>-613.54</v>
       </c>
     </row>
-    <row r="88" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A88" s="2">
         <v>45753.474710648145</v>
       </c>
@@ -4562,7 +4568,7 @@
         <v>-210</v>
       </c>
     </row>
-    <row r="89" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A89" s="2">
         <v>45753.473576388889</v>
       </c>
@@ -4603,7 +4609,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="90" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A90" s="2">
         <v>45753.473564814813</v>
       </c>
@@ -4647,7 +4653,7 @@
         <v>-210</v>
       </c>
     </row>
-    <row r="91" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>45752.947997685187</v>
       </c>
@@ -4691,7 +4697,7 @@
         <v>-4000</v>
       </c>
     </row>
-    <row r="92" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>45752.859305555554</v>
       </c>
@@ -4732,7 +4738,7 @@
         <v>-249.99</v>
       </c>
     </row>
-    <row r="93" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>45751.944837962961</v>
       </c>
@@ -4776,7 +4782,7 @@
         <v>-10000</v>
       </c>
     </row>
-    <row r="94" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>45751.925983796296</v>
       </c>
@@ -4817,7 +4823,7 @@
         <v>-1500</v>
       </c>
     </row>
-    <row r="95" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A95" s="2">
         <v>45751.863425925927</v>
       </c>
@@ -4858,7 +4864,7 @@
         <v>-264</v>
       </c>
     </row>
-    <row r="96" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>45751.86005787037</v>
       </c>
@@ -4899,7 +4905,7 @@
         <v>-1321.91</v>
       </c>
     </row>
-    <row r="97" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>45751.003865740742</v>
       </c>
@@ -4940,7 +4946,7 @@
         <v>-750</v>
       </c>
     </row>
-    <row r="98" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A98" s="2">
         <v>45750.940659722219</v>
       </c>
@@ -4978,7 +4984,7 @@
         <v>13.54</v>
       </c>
     </row>
-    <row r="99" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>45750.907754629632</v>
       </c>
@@ -5019,7 +5025,7 @@
         <v>-691.9</v>
       </c>
     </row>
-    <row r="100" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>45750.771886574075</v>
       </c>
@@ -5060,7 +5066,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="101" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A101" s="2">
         <v>45750.717488425929</v>
       </c>
@@ -5101,7 +5107,7 @@
         <v>-400</v>
       </c>
     </row>
-    <row r="102" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A102" s="2">
         <v>45750.674733796295</v>
       </c>
@@ -5145,7 +5151,7 @@
         <v>-210</v>
       </c>
     </row>
-    <row r="103" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>45750.654768518521</v>
       </c>
@@ -5189,7 +5195,7 @@
         <v>-999.8</v>
       </c>
     </row>
-    <row r="104" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A104" s="2">
         <v>45750.650023148148</v>
       </c>
@@ -5230,7 +5236,7 @@
         <v>1382.45</v>
       </c>
     </row>
-    <row r="105" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A105" s="2">
         <v>45750.650011574071</v>
       </c>
@@ -5274,7 +5280,7 @@
         <v>-1382.45</v>
       </c>
     </row>
-    <row r="106" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>45750.640219907407</v>
       </c>
@@ -5315,7 +5321,7 @@
         <v>-560</v>
       </c>
     </row>
-    <row r="107" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>45750.582118055558</v>
       </c>
@@ -5359,7 +5365,7 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="108" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A108" s="2">
         <v>45750.520254629628</v>
       </c>
@@ -5403,7 +5409,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="109" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A109" s="2">
         <v>45750.519513888888</v>
       </c>
@@ -5447,7 +5453,7 @@
         <v>-60</v>
       </c>
     </row>
-    <row r="110" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>45750.519201388888</v>
       </c>
@@ -5491,7 +5497,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="111" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A111" s="2">
         <v>45750.459618055553</v>
       </c>
@@ -5535,7 +5541,7 @@
         <v>-200</v>
       </c>
     </row>
-    <row r="112" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>45749.908159722225</v>
       </c>
@@ -5579,7 +5585,7 @@
         <v>-270</v>
       </c>
     </row>
-    <row r="113" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A113" s="2">
         <v>45749.821585648147</v>
       </c>
@@ -5620,7 +5626,7 @@
         <v>-150</v>
       </c>
     </row>
-    <row r="114" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>45749.641192129631</v>
       </c>
@@ -5664,7 +5670,7 @@
         <v>-396</v>
       </c>
     </row>
-    <row r="115" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>45749.58865740741</v>
       </c>
@@ -5702,7 +5708,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="116" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A116" s="2">
         <v>45749.584699074076</v>
       </c>
@@ -5746,7 +5752,7 @@
         <v>-500</v>
       </c>
     </row>
-    <row r="117" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A117" s="2">
         <v>45749.360532407409</v>
       </c>
@@ -5790,7 +5796,7 @@
         <v>-279.98</v>
       </c>
     </row>
-    <row r="118" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>45748.820752314816</v>
       </c>
@@ -5834,7 +5840,7 @@
         <v>-292.98</v>
       </c>
     </row>
-    <row r="119" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A119" s="2">
         <v>45748.794571759259</v>
       </c>
@@ -5878,7 +5884,7 @@
         <v>-210</v>
       </c>
     </row>
-    <row r="120" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>45748.668564814812</v>
       </c>
@@ -5922,7 +5928,7 @@
         <v>-248</v>
       </c>
     </row>
-    <row r="121" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A121" s="2">
         <v>45748.656053240738</v>
       </c>
@@ -5966,7 +5972,7 @@
         <v>-335</v>
       </c>
     </row>
-    <row r="122" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>45748.534560185188</v>
       </c>
@@ -6010,7 +6016,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="123" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A123" s="2">
         <v>45748.534155092595</v>
       </c>
@@ -6054,7 +6060,7 @@
         <v>-95</v>
       </c>
     </row>
-    <row r="124" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A124" s="2">
         <v>45748.416585648149</v>
       </c>
@@ -6098,7 +6104,7 @@
         <v>-299</v>
       </c>
     </row>
-    <row r="125" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>45748.401921296296</v>
       </c>
@@ -6136,7 +6142,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="126" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="2">
         <v>45748.396099537036</v>
       </c>
@@ -6177,6 +6183,182 @@
         <v>0</v>
       </c>
       <c r="O126" s="4">
+        <v>-625</v>
+      </c>
+    </row>
+    <row r="127" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A127" s="2">
+        <v>45717.396099537036</v>
+      </c>
+      <c r="B127" s="3">
+        <v>45748</v>
+      </c>
+      <c r="C127" t="s">
+        <v>15</v>
+      </c>
+      <c r="D127" t="s">
+        <v>16</v>
+      </c>
+      <c r="E127" s="4">
+        <v>-625</v>
+      </c>
+      <c r="F127" t="s">
+        <v>17</v>
+      </c>
+      <c r="G127" s="4">
+        <v>-625</v>
+      </c>
+      <c r="H127" t="s">
+        <v>17</v>
+      </c>
+      <c r="J127" t="s">
+        <v>18</v>
+      </c>
+      <c r="K127" t="s">
+        <v>118</v>
+      </c>
+      <c r="L127" t="s">
+        <v>119</v>
+      </c>
+      <c r="M127" s="4">
+        <v>0</v>
+      </c>
+      <c r="N127" s="4">
+        <v>0</v>
+      </c>
+      <c r="O127" s="4">
+        <v>-625</v>
+      </c>
+    </row>
+    <row r="128" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A128" s="2">
+        <v>45689.396099537036</v>
+      </c>
+      <c r="B128" s="3">
+        <v>45748</v>
+      </c>
+      <c r="C128" t="s">
+        <v>15</v>
+      </c>
+      <c r="D128" t="s">
+        <v>16</v>
+      </c>
+      <c r="E128" s="4">
+        <v>-625</v>
+      </c>
+      <c r="F128" t="s">
+        <v>17</v>
+      </c>
+      <c r="G128" s="4">
+        <v>-625</v>
+      </c>
+      <c r="H128" t="s">
+        <v>17</v>
+      </c>
+      <c r="J128" t="s">
+        <v>18</v>
+      </c>
+      <c r="K128" t="s">
+        <v>118</v>
+      </c>
+      <c r="L128" t="s">
+        <v>119</v>
+      </c>
+      <c r="M128" s="4">
+        <v>0</v>
+      </c>
+      <c r="N128" s="4">
+        <v>0</v>
+      </c>
+      <c r="O128" s="4">
+        <v>-625</v>
+      </c>
+    </row>
+    <row r="129" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A129" s="2">
+        <v>45658.396099537036</v>
+      </c>
+      <c r="B129" s="3">
+        <v>45748</v>
+      </c>
+      <c r="C129" t="s">
+        <v>15</v>
+      </c>
+      <c r="D129" t="s">
+        <v>16</v>
+      </c>
+      <c r="E129" s="4">
+        <v>-625</v>
+      </c>
+      <c r="F129" t="s">
+        <v>17</v>
+      </c>
+      <c r="G129" s="4">
+        <v>-625</v>
+      </c>
+      <c r="H129" t="s">
+        <v>17</v>
+      </c>
+      <c r="J129" t="s">
+        <v>18</v>
+      </c>
+      <c r="K129" t="s">
+        <v>118</v>
+      </c>
+      <c r="L129" t="s">
+        <v>119</v>
+      </c>
+      <c r="M129" s="4">
+        <v>0</v>
+      </c>
+      <c r="N129" s="4">
+        <v>0</v>
+      </c>
+      <c r="O129" s="4">
+        <v>-625</v>
+      </c>
+    </row>
+    <row r="130" spans="1:15" ht="16.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A130" s="2">
+        <v>45627.396099537036</v>
+      </c>
+      <c r="B130" s="3">
+        <v>45748</v>
+      </c>
+      <c r="C130" t="s">
+        <v>15</v>
+      </c>
+      <c r="D130" t="s">
+        <v>16</v>
+      </c>
+      <c r="E130" s="4">
+        <v>-625</v>
+      </c>
+      <c r="F130" t="s">
+        <v>17</v>
+      </c>
+      <c r="G130" s="4">
+        <v>-625</v>
+      </c>
+      <c r="H130" t="s">
+        <v>17</v>
+      </c>
+      <c r="J130" t="s">
+        <v>18</v>
+      </c>
+      <c r="K130" t="s">
+        <v>118</v>
+      </c>
+      <c r="L130" t="s">
+        <v>119</v>
+      </c>
+      <c r="M130" s="4">
+        <v>0</v>
+      </c>
+      <c r="N130" s="4">
+        <v>0</v>
+      </c>
+      <c r="O130" s="4">
         <v>-625</v>
       </c>
     </row>

</xml_diff>